<commit_message>
feat: distance neutral fallback, unmasked phone in full info modal, rich edit modal with map, and private shelter location in eye view only
</commit_message>
<xml_diff>
--- a/docs/Base de Datos de Masctoas.xlsx
+++ b/docs/Base de Datos de Masctoas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30411"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30412"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f5f906da8c23dd95/Desktop/Terremoto Mascotas/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3502" documentId="11_F25DC773A252ABDACC10485489D862385BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06DF067F-C0D0-40FE-B307-D64772C88131}"/>
+  <xr:revisionPtr revIDLastSave="3503" documentId="11_F25DC773A252ABDACC10485489D862385BDE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C866F318-2CE6-41C5-BE22-FA7CA74F75FB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="24" yWindow="0" windowWidth="23016" windowHeight="12216" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Observadas" sheetId="1" r:id="rId1"/>
@@ -3062,7 +3062,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3092,6 +3092,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -3110,26 +3123,23 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3152,27 +3162,15 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3192,6 +3190,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3490,7 +3492,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F944E3DE-FE9C-4E6E-B46E-81628292EFC9}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:V101"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3509,109 +3510,109 @@
     <col min="18" max="18" width="72" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="17.21875" hidden="1" customWidth="1"/>
     <col min="20" max="20" width="10" hidden="1" customWidth="1"/>
-    <col min="21" max="21" width="16.6640625" style="41" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19" t="s">
+      <c r="E1" s="13"/>
+      <c r="F1" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="19" t="s">
+      <c r="G1" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
-      <c r="P1" s="19"/>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="19" t="s">
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
+      <c r="O1" s="13"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="13"/>
+      <c r="R1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="S1" s="21" t="s">
+      <c r="S1" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="T1" s="19" t="s">
+      <c r="T1" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="U1" s="39" t="s">
+      <c r="U1" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="V1" s="20" t="s">
+      <c r="V1" s="15" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="2" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="19"/>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="22" t="s">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="G2" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="H2" s="20" t="s">
+      <c r="H2" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="20"/>
-      <c r="J2" s="20"/>
-      <c r="K2" s="20" t="s">
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="20" t="s">
+      <c r="L2" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="20" t="s">
+      <c r="M2" s="15" t="s">
         <v>66</v>
       </c>
-      <c r="N2" s="20" t="s">
+      <c r="N2" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="O2" s="20" t="s">
+      <c r="O2" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="P2" s="20" t="s">
+      <c r="P2" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="Q2" s="20" t="s">
+      <c r="Q2" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="R2" s="19"/>
-      <c r="S2" s="21"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="20"/>
-    </row>
-    <row r="3" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
+      <c r="R2" s="13"/>
+      <c r="S2" s="17"/>
+      <c r="T2" s="13"/>
+      <c r="U2" s="13"/>
+      <c r="V2" s="15"/>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
       <c r="D3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="19"/>
-      <c r="G3" s="22"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="14"/>
       <c r="H3" s="1" t="s">
         <v>28</v>
       </c>
@@ -3621,20 +3622,20 @@
       <c r="J3" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="20"/>
-      <c r="O3" s="20"/>
-      <c r="P3" s="20"/>
-      <c r="Q3" s="20"/>
-      <c r="R3" s="19"/>
-      <c r="S3" s="21"/>
-      <c r="T3" s="19"/>
-      <c r="U3" s="19"/>
-      <c r="V3" s="20"/>
-    </row>
-    <row r="4" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="15"/>
+      <c r="Q3" s="15"/>
+      <c r="R3" s="13"/>
+      <c r="S3" s="17"/>
+      <c r="T3" s="13"/>
+      <c r="U3" s="13"/>
+      <c r="V3" s="15"/>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
         <v>68</v>
       </c>
@@ -3700,7 +3701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
         <v>69</v>
       </c>
@@ -3766,7 +3767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>70</v>
       </c>
@@ -3832,7 +3833,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
         <v>71</v>
       </c>
@@ -3898,7 +3899,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
         <v>72</v>
       </c>
@@ -3964,7 +3965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A9" s="7" t="s">
         <v>73</v>
       </c>
@@ -4030,7 +4031,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
         <v>78</v>
       </c>
@@ -4096,7 +4097,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>86</v>
       </c>
@@ -4162,7 +4163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A12" s="7" t="s">
         <v>87</v>
       </c>
@@ -4228,7 +4229,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A13" s="7" t="s">
         <v>88</v>
       </c>
@@ -4353,14 +4354,14 @@
       <c r="T14" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="U14" s="40">
+      <c r="U14" s="4">
         <v>3022853805</v>
       </c>
       <c r="V14" s="7">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>90</v>
       </c>
@@ -4426,7 +4427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A16" s="7" t="s">
         <v>91</v>
       </c>
@@ -4492,7 +4493,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A17" s="7" t="s">
         <v>92</v>
       </c>
@@ -4558,7 +4559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A18" s="7" t="s">
         <v>93</v>
       </c>
@@ -4624,7 +4625,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A19" s="7" t="s">
         <v>94</v>
       </c>
@@ -4690,7 +4691,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A20" s="7" t="s">
         <v>95</v>
       </c>
@@ -4756,7 +4757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A21" s="7" t="s">
         <v>96</v>
       </c>
@@ -4822,7 +4823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A22" s="7" t="s">
         <v>97</v>
       </c>
@@ -4888,7 +4889,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>98</v>
       </c>
@@ -4954,7 +4955,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A24" s="7" t="s">
         <v>99</v>
       </c>
@@ -5020,7 +5021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A25" s="7" t="s">
         <v>100</v>
       </c>
@@ -5086,7 +5087,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A26" s="7" t="s">
         <v>101</v>
       </c>
@@ -5152,7 +5153,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
         <v>102</v>
       </c>
@@ -5218,7 +5219,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A28" s="7" t="s">
         <v>103</v>
       </c>
@@ -5284,7 +5285,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A29" s="7" t="s">
         <v>104</v>
       </c>
@@ -5350,7 +5351,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A30" s="7" t="s">
         <v>105</v>
       </c>
@@ -5416,7 +5417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A31" s="7" t="s">
         <v>106</v>
       </c>
@@ -5482,7 +5483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A32" s="7" t="s">
         <v>107</v>
       </c>
@@ -5548,7 +5549,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A33" s="7" t="s">
         <v>108</v>
       </c>
@@ -5614,7 +5615,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A34" s="7" t="s">
         <v>109</v>
       </c>
@@ -5680,7 +5681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A35" s="7" t="s">
         <v>110</v>
       </c>
@@ -5746,7 +5747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>111</v>
       </c>
@@ -5812,7 +5813,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A37" s="7" t="s">
         <v>112</v>
       </c>
@@ -5878,7 +5879,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A38" s="7" t="s">
         <v>113</v>
       </c>
@@ -5944,7 +5945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A39" s="7" t="s">
         <v>114</v>
       </c>
@@ -6010,7 +6011,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A40" s="7" t="s">
         <v>115</v>
       </c>
@@ -6076,7 +6077,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A41" s="7" t="s">
         <v>116</v>
       </c>
@@ -6142,7 +6143,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A42" s="7" t="s">
         <v>117</v>
       </c>
@@ -6208,7 +6209,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A43" s="7" t="s">
         <v>118</v>
       </c>
@@ -6274,7 +6275,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A44" s="7" t="s">
         <v>119</v>
       </c>
@@ -6340,7 +6341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A45" s="7" t="s">
         <v>120</v>
       </c>
@@ -6406,7 +6407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A46" s="7" t="s">
         <v>121</v>
       </c>
@@ -6472,7 +6473,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A47" s="7" t="s">
         <v>122</v>
       </c>
@@ -6538,7 +6539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A48" s="7" t="s">
         <v>123</v>
       </c>
@@ -6604,7 +6605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A49" s="7" t="s">
         <v>124</v>
       </c>
@@ -6670,7 +6671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A50" s="7" t="s">
         <v>125</v>
       </c>
@@ -6736,7 +6737,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A51" s="7" t="s">
         <v>126</v>
       </c>
@@ -6802,7 +6803,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A52" s="7" t="s">
         <v>127</v>
       </c>
@@ -6868,7 +6869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A53" s="7" t="s">
         <v>128</v>
       </c>
@@ -6934,7 +6935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A54" s="7" t="s">
         <v>129</v>
       </c>
@@ -7000,7 +7001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A55" s="7" t="s">
         <v>130</v>
       </c>
@@ -7066,7 +7067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A56" s="7" t="s">
         <v>131</v>
       </c>
@@ -7132,7 +7133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A57" s="7" t="s">
         <v>132</v>
       </c>
@@ -7198,7 +7199,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="58" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A58" s="7" t="s">
         <v>133</v>
       </c>
@@ -7264,7 +7265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A59" s="7" t="s">
         <v>134</v>
       </c>
@@ -7330,7 +7331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A60" s="7" t="s">
         <v>135</v>
       </c>
@@ -7396,7 +7397,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>136</v>
       </c>
@@ -7462,7 +7463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>137</v>
       </c>
@@ -7528,7 +7529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A63" s="7" t="s">
         <v>138</v>
       </c>
@@ -7594,7 +7595,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A64" s="7" t="s">
         <v>139</v>
       </c>
@@ -7660,7 +7661,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A65" s="7" t="s">
         <v>140</v>
       </c>
@@ -7726,7 +7727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A66" s="7" t="s">
         <v>141</v>
       </c>
@@ -7792,7 +7793,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A67" s="7" t="s">
         <v>142</v>
       </c>
@@ -7858,7 +7859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A68" s="7" t="s">
         <v>143</v>
       </c>
@@ -7924,7 +7925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A69" s="7" t="s">
         <v>144</v>
       </c>
@@ -7990,7 +7991,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A70" s="7" t="s">
         <v>145</v>
       </c>
@@ -8056,7 +8057,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="1:22" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A71" s="7" t="s">
         <v>146</v>
       </c>
@@ -8120,7 +8121,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A72" s="7" t="s">
         <v>147</v>
       </c>
@@ -8186,7 +8187,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A73" s="7" t="s">
         <v>148</v>
       </c>
@@ -8252,7 +8253,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A74" s="7" t="s">
         <v>149</v>
       </c>
@@ -8318,7 +8319,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="75" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A75" s="7" t="s">
         <v>469</v>
       </c>
@@ -8384,7 +8385,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="76" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A76" s="7" t="s">
         <v>497</v>
       </c>
@@ -8450,7 +8451,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="77" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A77" s="7" t="s">
         <v>498</v>
       </c>
@@ -8516,7 +8517,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="78" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A78" s="7" t="s">
         <v>499</v>
       </c>
@@ -8582,7 +8583,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A79" s="7" t="s">
         <v>500</v>
       </c>
@@ -8648,7 +8649,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="80" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A80" s="7" t="s">
         <v>501</v>
       </c>
@@ -8714,7 +8715,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="81" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A81" s="7" t="s">
         <v>502</v>
       </c>
@@ -8780,7 +8781,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="82" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A82" s="7" t="s">
         <v>503</v>
       </c>
@@ -8844,7 +8845,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="83" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A83" s="7" t="s">
         <v>504</v>
       </c>
@@ -8910,7 +8911,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="84" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A84" s="7" t="s">
         <v>505</v>
       </c>
@@ -8976,7 +8977,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="85" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A85" s="7" t="s">
         <v>506</v>
       </c>
@@ -9042,7 +9043,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="86" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A86" s="7" t="s">
         <v>507</v>
       </c>
@@ -9108,7 +9109,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="87" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A87" s="7" t="s">
         <v>565</v>
       </c>
@@ -9174,7 +9175,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="88" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A88" s="7" t="s">
         <v>566</v>
       </c>
@@ -9240,7 +9241,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="89" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A89" s="7" t="s">
         <v>567</v>
       </c>
@@ -9306,7 +9307,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="90" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A90" s="7" t="s">
         <v>568</v>
       </c>
@@ -9372,7 +9373,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="91" spans="1:22" ht="43.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:22" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A91" s="7" t="s">
         <v>569</v>
       </c>
@@ -9424,7 +9425,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A92" s="7" t="s">
         <v>590</v>
       </c>
@@ -9474,7 +9475,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A93" s="7" t="s">
         <v>593</v>
       </c>
@@ -9524,7 +9525,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="94" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A94" s="7" t="s">
         <v>597</v>
       </c>
@@ -9568,7 +9569,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="95" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A95" s="7" t="s">
         <v>601</v>
       </c>
@@ -9612,7 +9613,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="96" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A96" s="7" t="s">
         <v>605</v>
       </c>
@@ -9656,7 +9657,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="97" spans="1:22" ht="28.8" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A97" s="7" t="s">
         <v>609</v>
       </c>
@@ -9698,7 +9699,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="98" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A98" s="7" t="s">
         <v>615</v>
       </c>
@@ -9742,7 +9743,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="99" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A99" s="7" t="s">
         <v>622</v>
       </c>
@@ -9786,7 +9787,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="100" spans="1:22" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A100" s="7" t="s">
         <v>626</v>
       </c>
@@ -9867,7 +9868,7 @@
       </c>
       <c r="S101" s="4"/>
       <c r="T101" s="4"/>
-      <c r="U101" s="40">
+      <c r="U101" s="4">
         <v>3154975605</v>
       </c>
       <c r="V101" s="7">
@@ -9876,11 +9877,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:V101" xr:uid="{F944E3DE-FE9C-4E6E-B46E-81628292EFC9}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Candy"/>
-      </filters>
-    </filterColumn>
     <filterColumn colId="3" showButton="0"/>
     <filterColumn colId="6" showButton="0"/>
     <filterColumn colId="7" showButton="0"/>
@@ -9894,18 +9890,6 @@
     <filterColumn colId="15" showButton="0"/>
   </autoFilter>
   <mergeCells count="20">
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="D1:E2"/>
-    <mergeCell ref="F1:F3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="G1:Q1"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="Q2:Q3"/>
     <mergeCell ref="U1:U3"/>
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="M2:M3"/>
@@ -9914,6 +9898,18 @@
     <mergeCell ref="O2:O3"/>
     <mergeCell ref="R1:R3"/>
     <mergeCell ref="T1:T3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="G1:Q1"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="Q2:Q3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="D1:E2"/>
+    <mergeCell ref="F1:F3"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9934,70 +9930,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="13" t="s">
         <v>904</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="18" t="s">
         <v>908</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="18" t="s">
         <v>909</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="18" t="s">
         <v>910</v>
       </c>
-      <c r="F1" s="16" t="s">
+      <c r="F1" s="21" t="s">
         <v>905</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="18" t="s">
         <v>902</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="18" t="s">
         <v>903</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="18" t="s">
         <v>914</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="18" t="s">
         <v>915</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="18" t="s">
         <v>906</v>
       </c>
-      <c r="L1" s="16" t="s">
+      <c r="L1" s="21" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="19"/>
-      <c r="B2" s="19"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-      <c r="L2" s="17"/>
+      <c r="A2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="22"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A3" s="19"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="18"/>
-      <c r="G3" s="15"/>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="18"/>
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="20"/>
+      <c r="K3" s="20"/>
+      <c r="L3" s="23"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -10217,105 +10213,105 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26" t="s">
+      <c r="B1" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="26" t="s">
+      <c r="C1" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="29" t="s">
+      <c r="D1" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="30"/>
-      <c r="F1" s="26" t="s">
+      <c r="E1" s="34"/>
+      <c r="F1" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="G1" s="33" t="s">
+      <c r="G1" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="34"/>
-      <c r="M1" s="34"/>
-      <c r="N1" s="34"/>
-      <c r="O1" s="34"/>
-      <c r="P1" s="34"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="23" t="s">
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+      <c r="L1" s="25"/>
+      <c r="M1" s="25"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
+      <c r="P1" s="25"/>
+      <c r="Q1" s="26"/>
+      <c r="R1" s="37" t="s">
         <v>427</v>
       </c>
-      <c r="S1" s="26" t="s">
+      <c r="S1" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="T1" s="23" t="s">
+      <c r="T1" s="37" t="s">
         <v>39</v>
       </c>
-      <c r="U1" s="26" t="s">
+      <c r="U1" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="V1" s="16" t="s">
+      <c r="V1" s="21" t="s">
         <v>388</v>
       </c>
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A2" s="27"/>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="13" t="s">
+      <c r="A2" s="31"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="35"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="H2" s="36" t="s">
+      <c r="H2" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="37"/>
-      <c r="J2" s="38"/>
-      <c r="K2" s="16" t="s">
+      <c r="I2" s="28"/>
+      <c r="J2" s="29"/>
+      <c r="K2" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="16" t="s">
+      <c r="L2" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="16" t="s">
+      <c r="M2" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="N2" s="16" t="s">
+      <c r="N2" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="O2" s="16" t="s">
+      <c r="O2" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="P2" s="16" t="s">
+      <c r="P2" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="Q2" s="16" t="s">
+      <c r="Q2" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="R2" s="24"/>
-      <c r="S2" s="27"/>
-      <c r="T2" s="24"/>
-      <c r="U2" s="27"/>
-      <c r="V2" s="17"/>
+      <c r="R2" s="38"/>
+      <c r="S2" s="31"/>
+      <c r="T2" s="38"/>
+      <c r="U2" s="31"/>
+      <c r="V2" s="22"/>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
-      <c r="A3" s="28"/>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
+      <c r="A3" s="32"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
       <c r="D3" s="1" t="s">
         <v>12</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="28"/>
-      <c r="G3" s="15"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="20"/>
       <c r="H3" s="1" t="s">
         <v>28</v>
       </c>
@@ -10325,18 +10321,18 @@
       <c r="J3" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="K3" s="18"/>
-      <c r="L3" s="18"/>
-      <c r="M3" s="18"/>
-      <c r="N3" s="18"/>
-      <c r="O3" s="18"/>
-      <c r="P3" s="18"/>
-      <c r="Q3" s="18"/>
-      <c r="R3" s="25"/>
-      <c r="S3" s="28"/>
-      <c r="T3" s="25"/>
-      <c r="U3" s="28"/>
-      <c r="V3" s="18"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="23"/>
+      <c r="R3" s="39"/>
+      <c r="S3" s="32"/>
+      <c r="T3" s="39"/>
+      <c r="U3" s="32"/>
+      <c r="V3" s="23"/>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
@@ -17300,6 +17296,16 @@
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="R1:R3"/>
+    <mergeCell ref="S1:S3"/>
+    <mergeCell ref="T1:T3"/>
+    <mergeCell ref="U1:U3"/>
+    <mergeCell ref="V1:V3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:B3"/>
+    <mergeCell ref="C1:C3"/>
+    <mergeCell ref="D1:E2"/>
+    <mergeCell ref="F1:F3"/>
     <mergeCell ref="G1:Q1"/>
     <mergeCell ref="N2:N3"/>
     <mergeCell ref="O2:O3"/>
@@ -17310,16 +17316,6 @@
     <mergeCell ref="K2:K3"/>
     <mergeCell ref="L2:L3"/>
     <mergeCell ref="M2:M3"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:B3"/>
-    <mergeCell ref="C1:C3"/>
-    <mergeCell ref="D1:E2"/>
-    <mergeCell ref="F1:F3"/>
-    <mergeCell ref="R1:R3"/>
-    <mergeCell ref="S1:S3"/>
-    <mergeCell ref="T1:T3"/>
-    <mergeCell ref="U1:U3"/>
-    <mergeCell ref="V1:V3"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>